<commit_message>
change to fall 26
</commit_message>
<xml_diff>
--- a/assessment_schedule.xlsx
+++ b/assessment_schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xinchen/Documents/GitRepo/websites/csc110/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8396ECB-B455-0441-B2CB-B5D2D164F249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A3C16E0-CF19-1443-9BDE-B42955CA3C02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3540" yWindow="600" windowWidth="19780" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25980" yWindow="2580" windowWidth="19780" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -219,18 +219,17 @@
     <t>Quiz 12</t>
   </si>
   <si>
-    <t>6:00-8:00pm</t>
+    <t>3:30-5:30pm</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -320,13 +319,6 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -348,7 +340,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -364,8 +356,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -612,8 +602,8 @@
       <c r="B2" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="15">
-        <v>46037</v>
+      <c r="C2" s="2">
+        <v>46259</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>5</v>
@@ -626,8 +616,8 @@
       <c r="B3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="15">
-        <v>46044</v>
+      <c r="C3" s="2">
+        <v>46266</v>
       </c>
       <c r="D3" s="12" t="s">
         <v>5</v>
@@ -644,7 +634,7 @@
         <v>8</v>
       </c>
       <c r="C4" s="2">
-        <v>46045</v>
+        <v>46267</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>6</v>
@@ -658,8 +648,8 @@
       <c r="B5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="15">
-        <v>46049</v>
+      <c r="C5" s="2">
+        <v>46273</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>5</v>
@@ -673,8 +663,8 @@
       <c r="B6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="15">
-        <v>46050</v>
+      <c r="C6" s="2">
+        <v>46274</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>6</v>
@@ -687,8 +677,8 @@
       <c r="B7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="15">
-        <v>46050</v>
+      <c r="C7" s="2">
+        <v>46274</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>6</v>
@@ -701,8 +691,8 @@
       <c r="B8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="15">
-        <v>46052</v>
+      <c r="C8" s="2">
+        <v>46276</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>6</v>
@@ -715,8 +705,8 @@
       <c r="B9" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="15">
-        <v>46056</v>
+      <c r="C9" s="2">
+        <v>46280</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>5</v>
@@ -732,8 +722,8 @@
       <c r="B10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="15">
-        <v>46057</v>
+      <c r="C10" s="2">
+        <v>46281</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>6</v>
@@ -746,8 +736,8 @@
       <c r="B11" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="15">
-        <v>46057</v>
+      <c r="C11" s="2">
+        <v>46281</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>6</v>
@@ -760,8 +750,8 @@
       <c r="B12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="15">
-        <v>46059</v>
+      <c r="C12" s="2">
+        <v>46283</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>6</v>
@@ -774,8 +764,8 @@
       <c r="B13" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="15">
-        <v>46063</v>
+      <c r="C13" s="2">
+        <v>46287</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>5</v>
@@ -791,8 +781,8 @@
       <c r="B14" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="15">
-        <v>46064</v>
+      <c r="C14" s="2">
+        <v>46288</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>6</v>
@@ -805,8 +795,8 @@
       <c r="B15" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="15">
-        <v>46064</v>
+      <c r="C15" s="2">
+        <v>46288</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>6</v>
@@ -819,8 +809,8 @@
       <c r="B16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="15">
-        <v>46066</v>
+      <c r="C16" s="2">
+        <v>46290</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>6</v>
@@ -833,8 +823,8 @@
       <c r="B17" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="15">
-        <v>46070</v>
+      <c r="C17" s="2">
+        <v>45930</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>5</v>
@@ -850,8 +840,8 @@
       <c r="B18" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="15">
-        <v>46071</v>
+      <c r="C18" s="2">
+        <v>46295</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>6</v>
@@ -864,8 +854,8 @@
       <c r="B19" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="15">
-        <v>46071</v>
+      <c r="C19" s="2">
+        <v>46295</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>6</v>
@@ -878,8 +868,8 @@
       <c r="B20" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="15">
-        <v>46073</v>
+      <c r="C20" s="2">
+        <v>46297</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>6</v>
@@ -892,8 +882,8 @@
       <c r="B21" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="15">
-        <v>46077</v>
+      <c r="C21" s="2">
+        <v>46301</v>
       </c>
       <c r="D21" s="12" t="s">
         <v>5</v>
@@ -906,8 +896,8 @@
       <c r="B22" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="15">
-        <v>46080</v>
+      <c r="C22" s="2">
+        <v>46304</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>6</v>
@@ -920,8 +910,8 @@
       <c r="B23" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="15">
-        <v>46080</v>
+      <c r="C23" s="2">
+        <v>46304</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>6</v>
@@ -934,8 +924,8 @@
       <c r="B24" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="15">
-        <v>46083</v>
+      <c r="C24" s="2">
+        <v>46307</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>6</v>
@@ -948,8 +938,8 @@
       <c r="B25" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="15">
-        <v>46084</v>
+      <c r="C25" s="2">
+        <v>46308</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>5</v>
@@ -965,8 +955,8 @@
       <c r="B26" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C26" s="15">
-        <v>46085</v>
+      <c r="C26" s="2">
+        <v>46309</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>6</v>
@@ -979,8 +969,8 @@
       <c r="B27" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C27" s="15">
-        <v>46085</v>
+      <c r="C27" s="2">
+        <v>46309</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>6</v>
@@ -993,8 +983,8 @@
       <c r="B28" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C28" s="15">
-        <v>46087</v>
+      <c r="C28" s="2">
+        <v>46311</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>6</v>
@@ -1007,8 +997,8 @@
       <c r="B29" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C29" s="15">
-        <v>46098</v>
+      <c r="C29" s="2">
+        <v>46315</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>5</v>
@@ -1021,8 +1011,8 @@
       <c r="B30" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C30" s="15">
-        <v>46099</v>
+      <c r="C30" s="2">
+        <v>46316</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>6</v>
@@ -1035,8 +1025,8 @@
       <c r="B31" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C31" s="15">
-        <v>46099</v>
+      <c r="C31" s="2">
+        <v>46316</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>6</v>
@@ -1049,8 +1039,8 @@
       <c r="B32" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C32" s="15">
-        <v>46101</v>
+      <c r="C32" s="2">
+        <v>46318</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>6</v>
@@ -1063,8 +1053,8 @@
       <c r="B33" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="C33" s="15">
-        <v>46105</v>
+      <c r="C33" s="2">
+        <v>46322</v>
       </c>
       <c r="D33" s="11" t="s">
         <v>5</v>
@@ -1077,8 +1067,8 @@
       <c r="B34" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C34" s="15">
-        <v>46106</v>
+      <c r="C34" s="2">
+        <v>46323</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>6</v>
@@ -1091,8 +1081,8 @@
       <c r="B35" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C35" s="15">
-        <v>46112</v>
+      <c r="C35" s="2">
+        <v>46329</v>
       </c>
       <c r="D35" s="11" t="s">
         <v>5</v>
@@ -1105,8 +1095,8 @@
       <c r="B36" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C36" s="15">
-        <v>46113</v>
+      <c r="C36" s="2">
+        <v>46330</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>6</v>
@@ -1119,8 +1109,8 @@
       <c r="B37" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C37" s="15">
-        <v>46113</v>
+      <c r="C37" s="2">
+        <v>46330</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>6</v>
@@ -1133,8 +1123,8 @@
       <c r="B38" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C38" s="15">
-        <v>46115</v>
+      <c r="C38" s="2">
+        <v>46332</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>6</v>
@@ -1147,8 +1137,8 @@
       <c r="B39" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C39" s="15">
-        <v>46120</v>
+      <c r="C39" s="2">
+        <v>46337</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>6</v>
@@ -1161,8 +1151,8 @@
       <c r="B40" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C40" s="15">
-        <v>46120</v>
+      <c r="C40" s="2">
+        <v>46337</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>6</v>
@@ -1175,8 +1165,8 @@
       <c r="B41" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C41" s="15">
-        <v>46122</v>
+      <c r="C41" s="2">
+        <v>46339</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>6</v>
@@ -1189,8 +1179,8 @@
       <c r="B42" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="C42" s="15">
-        <v>46126</v>
+      <c r="C42" s="2">
+        <v>46343</v>
       </c>
       <c r="D42" s="12" t="s">
         <v>5</v>
@@ -1203,8 +1193,8 @@
       <c r="B43" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C43" s="15">
-        <v>46127</v>
+      <c r="C43" s="2">
+        <v>46344</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>6</v>
@@ -1218,8 +1208,8 @@
       <c r="B44" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C44" s="15">
-        <v>46127</v>
+      <c r="C44" s="2">
+        <v>46344</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>6</v>
@@ -1232,8 +1222,8 @@
       <c r="B45" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="C45" s="15">
-        <v>46129</v>
+      <c r="C45" s="2">
+        <v>46346</v>
       </c>
       <c r="D45" s="12" t="s">
         <v>6</v>
@@ -1246,8 +1236,8 @@
       <c r="B46" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="C46" s="16">
-        <v>46133</v>
+      <c r="C46" s="2">
+        <v>46350</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>5</v>
@@ -1260,8 +1250,8 @@
       <c r="B47" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C47" s="16">
-        <v>46134</v>
+      <c r="C47" s="2">
+        <v>46351</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>6</v>
@@ -1274,8 +1264,8 @@
       <c r="B48" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C48" s="16">
-        <v>46134</v>
+      <c r="C48" s="2">
+        <v>46351</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>6</v>
@@ -1288,8 +1278,8 @@
       <c r="B49" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="C49" s="16">
-        <v>46136</v>
+      <c r="C49" s="2">
+        <v>46357</v>
       </c>
       <c r="D49" s="12" t="s">
         <v>6</v>
@@ -1302,8 +1292,8 @@
       <c r="B50" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="C50" s="16">
-        <v>46140</v>
+      <c r="C50" s="2">
+        <v>46357</v>
       </c>
       <c r="D50" s="12" t="s">
         <v>5</v>
@@ -1316,8 +1306,8 @@
       <c r="B51" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="C51" s="16">
-        <v>46141</v>
+      <c r="C51" s="2">
+        <v>46360</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>6</v>
@@ -1332,8 +1322,8 @@
       <c r="B52" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="C52" s="16">
-        <v>46141</v>
+      <c r="C52" s="2">
+        <v>46360</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>6</v>
@@ -1346,8 +1336,8 @@
       <c r="B53" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="C53" s="16">
-        <v>46143</v>
+      <c r="C53" s="2">
+        <v>46363</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>6</v>
@@ -1360,10 +1350,10 @@
       <c r="B54" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="C54" s="16">
-        <v>46150</v>
-      </c>
-      <c r="D54" s="17" t="s">
+      <c r="C54" s="2">
+        <v>46367</v>
+      </c>
+      <c r="D54" s="15" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>